<commit_message>
Add SEIP flexible data capture app
</commit_message>
<xml_diff>
--- a/data/SEIP_Captured_Data.xlsx
+++ b/data/SEIP_Captured_Data.xlsx
@@ -5448,7 +5448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC1"/>
+  <dimension ref="A1:BC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="18" customWidth="1" style="6" min="1" max="11"/>
@@ -5731,6 +5731,67 @@
         <is>
           <t>gps_accuracy_meters</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="Q2" t="n">
+        <v>-26.27266487958484</v>
+      </c>
+      <c r="R2" t="n">
+        <v>27.82919982214795</v>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="X2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>browser_geolocation</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:37:44</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>2026-07-07T16:37:44</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>seip_admin</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>JS001</t>
+        </is>
+      </c>
+      <c r="BA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>-26.272665, 27.829200</t>
+        </is>
+      </c>
+      <c r="BC2" t="n">
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>